<commit_message>
docs: config for win
</commit_message>
<xml_diff>
--- a/src/demo_app/student_data.xlsx
+++ b/src/demo_app/student_data.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -492,6 +492,38 @@
       <c r="F2" t="inlineStr">
         <is>
           <t>2021DHHTTTO2-ĐH K16</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>2021604573</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Lê Thị Phương</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>20212025</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>25/06/2003</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Triệu Sơn - Thanh Hóa</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2021DHHTTTO2-K16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add final protection
</commit_message>
<xml_diff>
--- a/src/demo_app/student_data.xlsx
+++ b/src/demo_app/student_data.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -492,6 +492,134 @@
       <c r="F2" t="inlineStr">
         <is>
           <t>2021DHHTTTO2-ĐH K16</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>2021602195</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Dương Văn Dũng</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2021-2025</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>13/10/2003</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Lang Giang - Bắc Giang</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2021DHKTPMO2 - ĐHK16</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>2021604573</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Lê Thị Phương</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2021-2025</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>25/06/2003</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Triệu Sơn - Thanh Hóa</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2021DHHTTTO2-K16</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>2021603359</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Nguyễn Minh Hiếu</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2021-2025</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>18/04/2003</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Thái Bình - Thái Bình</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2021DHKTPMO3-ĐH K16</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>2021601774</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Nguyễn Quyết Thàng</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2021-2025</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>28/10/2003</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Thanh Hoa - Thanh Hoa</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2021 DHKTPMO2 - ĐH K16</t>
         </is>
       </c>
     </row>

</xml_diff>